<commit_message>
Add Vascular Surgery DOCX files with date-range variants and upload workbook for user 105084
- 1st 1st: dates Jan-Jun 2025, new reg nos
- 2nd 1st: dates Jan-Jun 2026, new reg nos
- 2nd 2nd: dates Jul-Sep 2026, new reg nos + upload workbook with results
</commit_message>
<xml_diff>
--- a/generated-data/copy data/2nd 2nd/BCPS_Patient_Management_TESTONLY_66_FRESH_2026-09-17.xlsx
+++ b/generated-data/copy data/2nd 2nd/BCPS_Patient_Management_TESTONLY_66_FRESH_2026-09-17.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="0" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet sheetId="1" name="DataEntry" state="visible" r:id="rId4"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="578">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1202" uniqueCount="576">
   <si>
     <t>ExternalRowId</t>
   </si>
@@ -1352,403 +1352,397 @@
     <t>SUCCESS</t>
   </si>
   <si>
-    <t>95998e25-1265-491a-a8f2-e30f986f17c9</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:47:51.471Z</t>
+    <t>e26c8e77-de3a-4d12-a9b0-22f7b69f3684</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:03:09.948Z</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>aea975f7-74b2-4db9-ba92-b8567e75a429</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:48:00.839Z</t>
-  </si>
-  <si>
-    <t>2ab3a4e3-4af2-4797-b662-bd6a3788ea59</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:48:10.150Z</t>
-  </si>
-  <si>
-    <t>5bf3217a-dc7f-4af8-9266-75e8a83585d9</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:48:20.170Z</t>
-  </si>
-  <si>
-    <t>0225be22-5480-4804-b290-4c1b6584d907</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:48:30.138Z</t>
-  </si>
-  <si>
-    <t>a2d2078b-2996-4b18-83ae-ce3c95a9c68d</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:48:39.469Z</t>
-  </si>
-  <si>
-    <t>fcc79871-78c7-4142-a457-d452a69a03e7</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:48:49.382Z</t>
-  </si>
-  <si>
-    <t>efc3d064-e1b9-4f16-bbb4-44f6c8b7ea0c</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:48:59.272Z</t>
-  </si>
-  <si>
-    <t>ffae0aa9-e82d-4ec0-8011-aa4d18803bf2</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:49:09.168Z</t>
-  </si>
-  <si>
-    <t>dcc81149-4c63-4ebd-82d4-0ac0deee8b63</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:49:18.221Z</t>
-  </si>
-  <si>
-    <t>729f89e0-9553-4040-bb09-3d12953ddf07</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:49:27.363Z</t>
-  </si>
-  <si>
-    <t>b6faeb77-62f4-4570-972b-7f2ed6f83696</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:49:37.023Z</t>
-  </si>
-  <si>
-    <t>1b86319c-0b24-4603-ba35-f5925475fb6a</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:49:46.314Z</t>
-  </si>
-  <si>
-    <t>faf3334b-b029-497d-af41-d336737c2131</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:49:55.554Z</t>
-  </si>
-  <si>
-    <t>40cb64cd-da80-45cc-be8f-c52f04eac245</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:50:06.759Z</t>
-  </si>
-  <si>
-    <t>995c7595-4572-43f3-81df-9aba49736d15</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:50:16.568Z</t>
-  </si>
-  <si>
-    <t>2b03f1fe-b75e-48e5-8efd-74b11f0d694d</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:50:25.971Z</t>
-  </si>
-  <si>
-    <t>4413cfb2-e495-4094-bbfb-68c33711bf0d</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:50:36.174Z</t>
-  </si>
-  <si>
-    <t>7ce99339-bcff-4c9f-a05b-cc5e5c1edd39</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:50:45.179Z</t>
-  </si>
-  <si>
-    <t>a03443a0-6f13-4184-9465-905c70fbb67a</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:50:54.330Z</t>
-  </si>
-  <si>
-    <t>c338c6ef-0438-4cc0-86ee-a095a06eaf60</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:51:04.383Z</t>
-  </si>
-  <si>
-    <t>2d1e88cf-2aa2-453b-8f8f-e3efeba9ef8f</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:51:13.473Z</t>
-  </si>
-  <si>
-    <t>c3fb058f-2a49-4112-930d-5ec68a245daf</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:51:24.277Z</t>
-  </si>
-  <si>
-    <t>e1ebf31b-67bf-46a2-a7ec-461c0650be01</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:51:33.836Z</t>
-  </si>
-  <si>
-    <t>2bd2ce88-a52e-448d-aab3-79d2004299e8</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:51:42.975Z</t>
-  </si>
-  <si>
-    <t>a653c301-0032-42e3-a164-48cb678a099f</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:51:52.835Z</t>
-  </si>
-  <si>
-    <t>9ba52c2a-2ea2-41ab-b266-572437393773</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:52:02.541Z</t>
-  </si>
-  <si>
-    <t>bb5d8b75-105e-4991-91ba-5a1b5af1c7c0</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:52:11.809Z</t>
-  </si>
-  <si>
-    <t>60316304-06b8-4a54-a905-1f1c34a18b13</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:52:20.875Z</t>
-  </si>
-  <si>
-    <t>26526b1f-a51a-456c-9a18-f0bee4caa883</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:52:30.067Z</t>
-  </si>
-  <si>
-    <t>857aa206-725d-4808-bfe8-88afd696ff59</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:52:40.569Z</t>
-  </si>
-  <si>
-    <t>514b3f7d-3db3-490a-b99b-9e5509c7399b</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:52:50.276Z</t>
-  </si>
-  <si>
-    <t>7a60982e-c241-43a0-8389-5fb35ec4a7aa</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:52:59.372Z</t>
-  </si>
-  <si>
-    <t>8d89f729-78b6-44f4-8042-5014d6f39b3a</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:53:08.965Z</t>
-  </si>
-  <si>
-    <t>e1e28a73-e1a3-4829-b5c4-dde26f642b47</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:53:18.669Z</t>
-  </si>
-  <si>
-    <t>e65fe31b-9b64-49c4-be23-6a7bde8a13cb</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:53:28.373Z</t>
-  </si>
-  <si>
-    <t>f26ab1a8-40ec-4b47-a46c-c5689db20891</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:53:37.486Z</t>
-  </si>
-  <si>
-    <t>b9f9ab84-77d9-430e-b1fc-d952a946ca5f</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:53:46.872Z</t>
-  </si>
-  <si>
-    <t>bdee9c53-15c2-4c00-b074-104c16288d34</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:53:56.075Z</t>
-  </si>
-  <si>
-    <t>51ae49a6-9bcd-4455-95c9-150cfe80e793</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:54:05.734Z</t>
-  </si>
-  <si>
-    <t>7dfbd29f-216d-4da9-86be-4954fec38043</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:54:14.770Z</t>
-  </si>
-  <si>
-    <t>1ae1a346-f600-49a9-8ee4-e554edae658f</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:54:24.674Z</t>
-  </si>
-  <si>
-    <t>1fe139fc-37ba-4534-b827-0fe87d2638fd</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:54:33.773Z</t>
-  </si>
-  <si>
-    <t>37f58f14-b76f-4bdf-8bbf-8c3fde20d2d0</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:54:42.971Z</t>
-  </si>
-  <si>
-    <t>d464ff02-1bdf-47f9-8057-fd833dda9a57</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:54:52.372Z</t>
-  </si>
-  <si>
-    <t>1fe7e1de-c057-4cea-83e2-27c5d2af7987</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:55:01.936Z</t>
-  </si>
-  <si>
-    <t>b0de5503-07de-4082-b3e6-8539a45cf859</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:55:12.586Z</t>
-  </si>
-  <si>
-    <t>c14c13a3-147a-41c9-a85b-0483ca83e535</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:55:22.578Z</t>
-  </si>
-  <si>
-    <t>2aea6f47-8d11-41ef-b93e-f35fd0c7ad6d</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:55:32.581Z</t>
-  </si>
-  <si>
-    <t>8edaec7a-0f7f-4a74-98d1-94585e53e654</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:55:41.632Z</t>
-  </si>
-  <si>
-    <t>c0a00745-ebc4-45f8-8cc9-e93395eab07b</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:55:52.484Z</t>
-  </si>
-  <si>
-    <t>3df92b61-ae11-47e6-b66f-4dcfb98dd0c1</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:56:02.177Z</t>
-  </si>
-  <si>
-    <t>fc3ce5d2-6c6d-4ef8-8da8-b6776151c117</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:56:11.282Z</t>
-  </si>
-  <si>
-    <t>04c489f5-b9f3-4c06-9e41-a0e68ac08e9f</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:56:21.137Z</t>
-  </si>
-  <si>
-    <t>f797c0f6-cb56-4af4-9edf-fe4f515efae0</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:56:30.975Z</t>
-  </si>
-  <si>
-    <t>b6169a83-dedd-4d87-90e2-3a7e3171680b</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:56:40.233Z</t>
-  </si>
-  <si>
-    <t>7702786c-efa7-4af4-951a-c3b804c42bc8</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:56:49.375Z</t>
-  </si>
-  <si>
-    <t>3b7652cf-725a-4218-8fbd-a00d39bc4fba</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:56:58.739Z</t>
-  </si>
-  <si>
-    <t>e8ad461d-1286-448d-b501-3f7f992e3038</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:57:08.674Z</t>
-  </si>
-  <si>
-    <t>3512d48c-173c-4355-9f4f-f2c1ee88ddf9</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:57:17.929Z</t>
-  </si>
-  <si>
-    <t>5158e961-4c6d-4c36-b2ee-f23daf93b9f1</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:57:27.077Z</t>
-  </si>
-  <si>
-    <t>80c9a011-6bc2-4014-a356-5f1f676bc4d5</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:57:37.571Z</t>
-  </si>
-  <si>
-    <t>f5c4acd6-9de8-4521-a0d2-4ce39a6b7c54</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:57:47.273Z</t>
-  </si>
-  <si>
-    <t>10cc6074-b674-4450-a405-31431f0eb22b</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:57:57.080Z</t>
-  </si>
-  <si>
-    <t>1d295b0d-29de-40cc-ab71-9780c563814d</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:58:07.938Z</t>
-  </si>
-  <si>
-    <t>4abeae58-01bb-4a30-81db-b3a688085430</t>
-  </si>
-  <si>
-    <t>2026-09-23T08:58:17.176Z</t>
+    <t>70b374fb-9451-4f9d-82c9-f322911f8760</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:03:19.210Z</t>
+  </si>
+  <si>
+    <t>6ac2698f-2962-464f-bf35-2cdd430ba543</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:03:29.039Z</t>
+  </si>
+  <si>
+    <t>c81f8174-d077-4569-9160-c573b9c6b8c3</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:03:38.814Z</t>
+  </si>
+  <si>
+    <t>b9023078-b7fc-488c-a1c7-2a3e3fc14e8c</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:03:48.756Z</t>
+  </si>
+  <si>
+    <t>f6b89c7d-fa46-4538-8839-2fe3c57b8171</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:03:58.347Z</t>
+  </si>
+  <si>
+    <t>7345c4a0-058c-4c34-af24-0a89e9cb2872</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:04:07.260Z</t>
+  </si>
+  <si>
+    <t>abb58e7f-d0cb-4693-bcdf-a9f412ab1dce</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:04:16.600Z</t>
+  </si>
+  <si>
+    <t>ba9b67cd-4ac5-4575-90b7-1d4f4fcf578c</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:04:26.458Z</t>
+  </si>
+  <si>
+    <t>a71fcb0f-c62d-4278-b746-182033188121</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:04:36.199Z</t>
+  </si>
+  <si>
+    <t>263d1b24-e7ff-44be-8d38-874a99041a6d</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:04:46.002Z</t>
+  </si>
+  <si>
+    <t>11ba015f-c239-4e2a-a32c-a3c63517e3b3</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:04:55.000Z</t>
+  </si>
+  <si>
+    <t>d36891ee-3b0f-4fe8-8577-49eaf60bf662</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:05:04.798Z</t>
+  </si>
+  <si>
+    <t>278f5a29-647b-4596-a0a1-04ed0b9efc34</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:05:13.958Z</t>
+  </si>
+  <si>
+    <t>7a5d2b35-0d25-4d31-b2b8-0685ee475159</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:05:23.808Z</t>
+  </si>
+  <si>
+    <t>55d2ae04-e2fb-4eab-afa3-3588c8fbc1b4</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:05:32.998Z</t>
+  </si>
+  <si>
+    <t>667b26b3-638e-4f38-9f1c-0a61bdae6b12</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:05:42.042Z</t>
+  </si>
+  <si>
+    <t>9acf823f-74cf-40bc-8189-31e0bc90fa56</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:05:51.242Z</t>
+  </si>
+  <si>
+    <t>700a8b13-99ab-4257-8c1f-76175aa1bd9d</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:06:01.001Z</t>
+  </si>
+  <si>
+    <t>9bd4662d-c533-4892-989d-c0da3d682b2a</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:06:10.741Z</t>
+  </si>
+  <si>
+    <t>7dba0cee-d6c5-4540-887f-b813eb3be20a</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:06:19.802Z</t>
+  </si>
+  <si>
+    <t>8d7e180a-7bc7-4235-9d24-482bf54f3cc8</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:06:29.642Z</t>
+  </si>
+  <si>
+    <t>4ee07463-6fde-4060-a006-ad754412b49a</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:06:39.340Z</t>
+  </si>
+  <si>
+    <t>96490b86-3bfc-47ef-917f-9a963030fda1</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:06:49.102Z</t>
+  </si>
+  <si>
+    <t>a4f4d556-8e6b-42a5-8e85-70ecc9ca6afb</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:06:58.143Z</t>
+  </si>
+  <si>
+    <t>978abf1f-63b2-4682-9170-e8156131dd7f</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:07:07.344Z</t>
+  </si>
+  <si>
+    <t>d21885b2-93c6-4237-a64a-3bd082c1e3ef</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:07:16.445Z</t>
+  </si>
+  <si>
+    <t>67fe7d9d-5207-470d-b616-6f21d746b325</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:07:26.306Z</t>
+  </si>
+  <si>
+    <t>76b31a56-5a7b-46d7-a482-5a8fe7851634</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:07:35.245Z</t>
+  </si>
+  <si>
+    <t>cc33c06f-7eab-400b-8543-62839eaaa5a2</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:07:44.204Z</t>
+  </si>
+  <si>
+    <t>01dc21d8-7223-483c-9651-93200f2d02f0</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:07:54.102Z</t>
+  </si>
+  <si>
+    <t>0ca9e1ef-ed90-4160-a806-87797e533691</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:08:03.654Z</t>
+  </si>
+  <si>
+    <t>73d82bd3-f9de-40db-ab59-3d09665f2385</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:08:12.801Z</t>
+  </si>
+  <si>
+    <t>ed1e4d51-2f47-40cf-85e0-3e9631f4a3b5</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:08:22.983Z</t>
+  </si>
+  <si>
+    <t>8dffcd00-dafa-4e78-b602-c7821cf6f935</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:08:33.644Z</t>
+  </si>
+  <si>
+    <t>f3071d6c-b3a2-4271-aef7-925c10bb15b2</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:08:42.744Z</t>
+  </si>
+  <si>
+    <t>1c1fd55c-a9ff-4735-bb3e-777239a507dc</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:08:51.904Z</t>
+  </si>
+  <si>
+    <t>13e1f0c2-7bf4-4562-8426-05358640e98b</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:09:01.711Z</t>
+  </si>
+  <si>
+    <t>26e0e3b8-2922-440b-a6c5-784bb2e06ae3</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:09:11.402Z</t>
+  </si>
+  <si>
+    <t>b44edb3b-29a5-4fb5-96d6-1e2888b2027d</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:09:20.505Z</t>
+  </si>
+  <si>
+    <t>eafe1b35-976c-44eb-889b-71b7b790ace9</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:09:30.246Z</t>
+  </si>
+  <si>
+    <t>1c35ccd0-db33-4119-ad2b-d6e4c9432b12</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:09:39.200Z</t>
+  </si>
+  <si>
+    <t>313ee7a2-cf91-4ab9-8066-8c030bdc1775</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:09:48.505Z</t>
+  </si>
+  <si>
+    <t>f6144d17-f5b1-4772-aa08-3983477f0a30</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:09:58.146Z</t>
+  </si>
+  <si>
+    <t>ecf58730-4590-4e5d-95f7-a10ec430bc69</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:10:07.348Z</t>
+  </si>
+  <si>
+    <t>cc116355-22a6-44eb-8b02-5a9a1f65f03a</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:10:17.303Z</t>
+  </si>
+  <si>
+    <t>6c7e9210-3fde-42bb-93ac-93a15cd7bbae</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:10:27.050Z</t>
+  </si>
+  <si>
+    <t>21e6b7ec-748c-4f37-91a3-0dfde2c8d417</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:10:36.211Z</t>
+  </si>
+  <si>
+    <t>b03cfba9-593c-4a36-8b15-f8ade443e27f</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:10:45.504Z</t>
+  </si>
+  <si>
+    <t>ea92692e-2a9f-421e-8707-106904b35d00</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:10:55.106Z</t>
+  </si>
+  <si>
+    <t>31a430b2-5161-46a8-aa9b-0da04bb50ac3</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:11:04.151Z</t>
+  </si>
+  <si>
+    <t>e28a3870-2b99-49cc-97d1-7fc971802f3c</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:11:13.406Z</t>
+  </si>
+  <si>
+    <t>0eae9608-a261-4b8f-a22c-53327fb20e9a</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:11:23.050Z</t>
+  </si>
+  <si>
+    <t>da554e1a-4725-4f69-8eee-0454dfc7df19</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:11:32.308Z</t>
+  </si>
+  <si>
+    <t>dfe9131c-1ffa-465c-9ce4-5b170d969c6e</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:11:42.148Z</t>
+  </si>
+  <si>
+    <t>62b2c622-0017-4dd0-a1eb-dbfd21c9bbf0</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:11:51.805Z</t>
+  </si>
+  <si>
+    <t>94892a40-f92b-406e-a3b0-d614e181c1f7</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:12:00.852Z</t>
+  </si>
+  <si>
+    <t>245c3bd5-e450-4054-82b0-ff18fba37457</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:12:10.015Z</t>
+  </si>
+  <si>
+    <t>ae6db8ed-c8f2-4fe8-9a37-30322b932d9e</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:12:19.350Z</t>
+  </si>
+  <si>
+    <t>fca38288-f93b-444c-9b74-7e3ccc3b1962</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:12:29.150Z</t>
+  </si>
+  <si>
+    <t>a5cf5350-3edc-478d-8748-8baf2c806de6</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:12:39.148Z</t>
+  </si>
+  <si>
+    <t>288a8f30-b80c-4b54-a863-dacc6464b69a</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:12:48.511Z</t>
+  </si>
+  <si>
+    <t>cc8100f4-91b7-4cd6-9b1a-4fd0c2aa0432</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:12:57.746Z</t>
+  </si>
+  <si>
+    <t>4168bb68-2921-42fb-b14b-db572ab48ed0</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:13:07.505Z</t>
+  </si>
+  <si>
+    <t>78af43f8-d5f8-4031-bd81-233e1fabbe39</t>
+  </si>
+  <si>
+    <t>2026-10-01T04:13:17.209Z</t>
   </si>
 </sst>
 </file>
@@ -2125,11 +2119,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
   <dimension ref="A1:M67"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -4490,11 +4481,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:H67"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
+  <dimension ref="A1:H66"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="19.42578125" customWidth="1"/>
   </cols>
@@ -6215,32 +6203,6 @@
         <v>447</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>431</v>
-      </c>
-      <c r="B67">
-        <v>67</v>
-      </c>
-      <c r="C67" t="s">
-        <v>444</v>
-      </c>
-      <c r="D67" t="s">
-        <v>576</v>
-      </c>
-      <c r="E67" t="s">
-        <v>577</v>
-      </c>
-      <c r="F67" t="s">
-        <v>447</v>
-      </c>
-      <c r="G67" t="s">
-        <v>447</v>
-      </c>
-      <c r="H67" t="s">
-        <v>447</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>